<commit_message>
Add backtest scripts, refresh FO universe, update monitors and data - 2026-05-29
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-04.xlsx
+++ b/data/nifty_options/nifty_options_2026-04.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2075,6 +2075,474 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>10:00:31</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>24101.3</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>18.77</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24101.30 above TC 23935.24 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24101.30 above TC 23935.24 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>10:00:20</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>24156.3</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24156.30 above TC 24072.95 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24156.30 above TC 24072.95 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>10:00:20</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>24175.1</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24175.10 above TC 24020.28 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24175.10 above TC 24020.28 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>10:00:26</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>23878.85</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>18.72</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23878.85 below BC 24197.33 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23878.85 below BC 24197.33 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>